<commit_message>
Marathonplan: Mittwoch gedeckelt, damit Mo und Mi kurz bleiben
Der Qualitaetslauf am Mittwoch war in 32 Wochen laenger als der
Montag, bis zu 12 km. Ein- und Auslaufen gekuerzt und Wiederholungen
reduziert: Mittwoch jetzt hoechstens Montag + 2 km und nie ueber
10 km, in jeder Woche kuerzer als der lange Lauf am Freitag.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FUsfYuQHH2s6DefiNFEi2C
</commit_message>
<xml_diff>
--- a/marathonplan/Marathonplan_2026_2027.xlsx
+++ b/marathonplan/Marathonplan_2026_2027.xlsx
@@ -2342,7 +2342,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9.1</v>
+        <v>7.7</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>11</v>
@@ -2393,7 +2393,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5× 1000 m @ 5:40</t>
+          <t>4× 1000 m @ 5:40</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>4× 400 m Trab @ 7:30</t>
+          <t>3× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -2529,11 +2529,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -2603,7 +2599,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -2626,7 +2622,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -2645,7 +2641,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -2658,11 +2654,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>
@@ -2881,7 +2873,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10.2</v>
+        <v>7.1</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>12</v>
@@ -2905,7 +2897,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:10</t>
+          <t>1,5 km einlaufen @ 7:10</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -2932,7 +2924,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>3× 2000 m @ 5:45</t>
+          <t>2× 2000 m @ 5:45</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -2959,7 +2951,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>2× 600 m Trab @ 7:30</t>
+          <t>1× 600 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -3013,7 +3005,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -3036,7 +3028,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -3055,7 +3047,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -3068,11 +3060,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -3142,7 +3130,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -3165,7 +3153,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -3184,7 +3172,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -3197,11 +3185,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>
@@ -4474,7 +4458,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8.5</v>
+        <v>7</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>13</v>
@@ -4498,7 +4482,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:10</t>
+          <t>1,5 km einlaufen @ 7:10</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -4525,7 +4509,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5 km @ 5:35 (Tempolauf)</t>
+          <t>4 km @ 5:35 (Tempolauf)</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -4606,7 +4590,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -4629,7 +4613,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -4648,7 +4632,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -4661,11 +4645,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -4735,7 +4715,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -4758,7 +4738,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -4777,7 +4757,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -4790,11 +4770,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>
@@ -5013,7 +4989,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>13</v>
@@ -5037,7 +5013,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:10</t>
+          <t>1,5 km einlaufen @ 7:10</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -5064,7 +5040,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5× 1000 m @ 5:30</t>
+          <t>4× 1000 m @ 5:30</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -5091,7 +5067,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>4× 400 m Trab @ 7:30</t>
+          <t>3× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -5552,7 +5528,7 @@
         <v>5</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>7.7</v>
+        <v>6.3</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>10</v>
@@ -5603,7 +5579,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>4× 1000 m @ 5:30</t>
+          <t>3× 1000 m @ 5:30</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -5630,7 +5606,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>3× 400 m Trab @ 7:30</t>
+          <t>2× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -6075,7 +6051,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>13</v>
@@ -6099,7 +6075,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:05</t>
+          <t>1,5 km einlaufen @ 7:05</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -6614,7 +6590,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>11.5</v>
+        <v>9.1</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>14</v>
@@ -6638,7 +6614,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:05</t>
+          <t>1,5 km einlaufen @ 7:05</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -6665,7 +6641,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>6× 1000 m @ 5:25</t>
+          <t>5× 1000 m @ 5:25</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -6692,7 +6668,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>5× 400 m Trab @ 7:30</t>
+          <t>4× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -6719,7 +6695,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>1,5 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -7656,7 +7632,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>16</v>
@@ -7680,7 +7656,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:05</t>
+          <t>1,5 km einlaufen @ 7:05</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -7707,7 +7683,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>2× 3000 m @ 5:30</t>
+          <t>2× 2500 m @ 5:30</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -7761,7 +7737,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>1,5 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -12479,7 +12455,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>21</v>
@@ -12503,7 +12479,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:00</t>
+          <t>1,5 km einlaufen @ 7:00</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -12530,7 +12506,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5× 1000 m @ 5:35</t>
+          <t>4× 1000 m @ 5:35</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -12557,7 +12533,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>4× 400 m Trab @ 7:30</t>
+          <t>3× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -15278,7 +15254,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>22</v>
@@ -15302,7 +15278,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 7:00</t>
+          <t>1,5 km einlaufen @ 7:00</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -15329,7 +15305,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>8 km @ 6:24 (Marathon-Pace)</t>
+          <t>6 km @ 6:24 (Marathon-Pace)</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -15356,7 +15332,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1,5 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -15490,7 +15466,7 @@
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>Gel 25 g KH alle 20 min (75 g KH/h)</t>
+          <t>Wasser 400 ml</t>
         </is>
       </c>
       <c r="D14" s="33" t="inlineStr">
@@ -15507,11 +15483,7 @@
     <row r="15" ht="15.5" customHeight="1">
       <c r="A15" s="35" t="n"/>
       <c r="B15" s="36" t="inlineStr"/>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>Wasser 300 ml/h</t>
-        </is>
-      </c>
+      <c r="C15" s="36" t="inlineStr"/>
       <c r="D15" s="36" t="inlineStr">
         <is>
           <t>Elektrolytgetränk 500 ml/h (Natrium)</t>
@@ -20780,7 +20752,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>13</v>
@@ -20804,7 +20776,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -20831,7 +20803,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5× 1000 m @ 4:55</t>
+          <t>4× 1000 m @ 4:55</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -20858,7 +20830,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>4× 400 m Trab @ 7:30</t>
+          <t>3× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -21890,7 +21862,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>11.5</v>
+        <v>9.1</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>13</v>
@@ -21914,7 +21886,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -21941,7 +21913,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>6× 1000 m @ 4:50</t>
+          <t>5× 1000 m @ 4:50</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -21968,7 +21940,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>5× 400 m Trab @ 7:30</t>
+          <t>4× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -21995,7 +21967,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>1,5 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -23008,7 +22980,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9.800000000000001</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>14</v>
@@ -23032,7 +23004,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -23113,7 +23085,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1,5 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -23571,7 +23543,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>9.6</v>
+        <v>7.7</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>12</v>
@@ -23622,7 +23594,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>5× 1000 m @ 4:50</t>
+          <t>4× 1000 m @ 4:50</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -23649,7 +23621,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>4× 400 m Trab @ 7:30</t>
+          <t>3× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -23676,7 +23648,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>1,5 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -23703,7 +23675,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -23726,7 +23698,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -23745,7 +23717,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -23758,11 +23730,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -23832,7 +23800,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -23855,7 +23823,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -23874,7 +23842,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -23887,11 +23855,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>
@@ -24134,7 +24098,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>14</v>
@@ -24158,7 +24122,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -24239,7 +24203,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -24266,7 +24230,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -24289,7 +24253,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -24308,7 +24272,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -24321,11 +24285,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -24395,7 +24355,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -24418,7 +24378,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -24437,7 +24397,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -24450,11 +24410,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>
@@ -24697,7 +24653,7 @@
         <v>8</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>14</v>
@@ -24721,7 +24677,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -24802,7 +24758,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1,5 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -26338,7 +26294,7 @@
         <v>7</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>12</v>
+        <v>9.1</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>14</v>
@@ -26362,7 +26318,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -26389,7 +26345,7 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>6× 1000 m @ 4:45</t>
+          <t>5× 1000 m @ 4:45</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
@@ -26416,7 +26372,7 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>5× 400 m Trab @ 7:30</t>
+          <t>4× 400 m Trab @ 7:30</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
@@ -26443,7 +26399,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -26901,7 +26857,7 @@
         <v>6</v>
       </c>
       <c r="C5" s="31" t="n">
-        <v>8.6</v>
+        <v>7.6</v>
       </c>
       <c r="D5" s="31" t="n">
         <v>10</v>
@@ -26925,7 +26881,7 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>2 km einlaufen @ 6:55</t>
+          <t>1,5 km einlaufen @ 6:55</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
@@ -27006,7 +26962,7 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>2 km auslaufen @ 7:30</t>
+          <t>1,5 km auslaufen @ 7:30</t>
         </is>
       </c>
       <c r="D9" s="15" t="inlineStr">
@@ -27033,7 +26989,7 @@
       </c>
       <c r="C10" s="33" t="inlineStr">
         <is>
-          <t>Haferflocken 80 g (2–3 h vorher)</t>
+          <t>Banane 120 g (1,5 h vorher)</t>
         </is>
       </c>
       <c r="D10" s="33" t="inlineStr">
@@ -27056,7 +27012,7 @@
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
-          <t>Banane 120 g</t>
+          <t>Maiswaffel 2 Stück (14 g)</t>
         </is>
       </c>
       <c r="D11" s="36" t="inlineStr">
@@ -27075,7 +27031,7 @@
       </c>
       <c r="C12" s="36" t="inlineStr">
         <is>
-          <t>Datteln 40 g</t>
+          <t>Wasser 300 ml</t>
         </is>
       </c>
       <c r="D12" s="36" t="inlineStr">
@@ -27088,11 +27044,7 @@
     <row r="13" ht="15.5" customHeight="1">
       <c r="A13" s="38" t="n"/>
       <c r="B13" s="39" t="inlineStr"/>
-      <c r="C13" s="39" t="inlineStr">
-        <is>
-          <t>Wasser 500 ml</t>
-        </is>
-      </c>
+      <c r="C13" s="39" t="inlineStr"/>
       <c r="D13" s="39" t="inlineStr">
         <is>
           <t>Wasser 500 ml</t>
@@ -27154,7 +27106,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>Clear Protein 40 g in 500 ml Wasser</t>
+          <t>Clear Protein 30 g in 400 ml Wasser</t>
         </is>
       </c>
       <c r="D17" s="33" t="inlineStr">
@@ -27177,7 +27129,7 @@
       </c>
       <c r="C18" s="36" t="inlineStr">
         <is>
-          <t>Banane 2 Stück (240 g)</t>
+          <t>Banane 1 Stück (120 g)</t>
         </is>
       </c>
       <c r="D18" s="36" t="inlineStr">
@@ -27196,7 +27148,7 @@
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
-          <t>Maiswaffel 4 Stück (28 g)</t>
+          <t>Reiswaffel 3 Stück (27 g)</t>
         </is>
       </c>
       <c r="D19" s="36" t="inlineStr">
@@ -27209,11 +27161,7 @@
     <row r="20" ht="15.5" customHeight="1">
       <c r="A20" s="38" t="n"/>
       <c r="B20" s="39" t="inlineStr"/>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>Datteln 20 g</t>
-        </is>
-      </c>
+      <c r="C20" s="39" t="inlineStr"/>
       <c r="D20" s="39" t="inlineStr">
         <is>
           <t>Datteln 20 g</t>

</xml_diff>

<commit_message>
Wings for Life als viertes Ziel
Der Lauf am 09.05.2027 stand nur in Woche 33, nicht unter den Zielen.
Jetzt vier Rennen, chronologisch: Halbmarathon, Wings for Life,
Marathon, 5,7 km. Traumziel "bis zur Einholung", Einschaetzung
19,33 km bei 5:44/km. Dazu eine Hinweiszeile mit Startzeit, Startort
und den Stufen des Catcher Car.

Gilt fuer die Excel-Datei und fuer die Ziele der laufen-App - beide
kommen aus derselben Quelle.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FUsfYuQHH2s6DefiNFEi2C
</commit_message>
<xml_diff>
--- a/marathonplan/Marathonplan_2026_2027.xlsx
+++ b/marathonplan/Marathonplan_2026_2027.xlsx
@@ -853,7 +853,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K35"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -884,7 +884,8 @@
       </c>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="n"/>
-      <c r="D3" s="4" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="4" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
@@ -899,10 +900,15 @@
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
+          <t>Wings for Life</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
           <t>Marathon</t>
         </is>
       </c>
-      <c r="D4" s="7" t="inlineStr">
+      <c r="E4" s="7" t="inlineStr">
         <is>
           <t>5,7 km</t>
         </is>
@@ -921,10 +927,15 @@
       </c>
       <c r="C5" s="9" t="inlineStr">
         <is>
+          <t>09.05.2027</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr">
+        <is>
           <t>23.05.2027</t>
         </is>
       </c>
-      <c r="D5" s="10" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>16.09.2027</t>
         </is>
@@ -943,10 +954,15 @@
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
+          <t>Wien</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
           <t>Salzburg</t>
         </is>
       </c>
-      <c r="D6" s="10" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>Salzburg</t>
         </is>
@@ -965,10 +981,15 @@
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
+          <t>Woche 33</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr">
+        <is>
           <t>Woche 35</t>
         </is>
       </c>
-      <c r="D7" s="10" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>Woche 52</t>
         </is>
@@ -987,10 +1008,15 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
+          <t>bis zur Einholung</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
           <t>3:59:59</t>
         </is>
       </c>
-      <c r="D8" s="10" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>24:59</t>
         </is>
@@ -1009,10 +1035,15 @@
       </c>
       <c r="C9" s="9" t="inlineStr">
         <is>
+          <t>5:44/km</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
           <t>5:41/km</t>
         </is>
       </c>
-      <c r="D9" s="10" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>4:23/km</t>
         </is>
@@ -1031,10 +1062,15 @@
       </c>
       <c r="C10" s="9" t="inlineStr">
         <is>
+          <t>19,33 km</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
           <t>4:30:00</t>
         </is>
       </c>
-      <c r="D10" s="10" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>26:00</t>
         </is>
@@ -1053,10 +1089,15 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
+          <t>5:44/km</t>
+        </is>
+      </c>
+      <c r="D11" s="9" t="inlineStr">
+        <is>
           <t>6:24/km</t>
         </is>
       </c>
-      <c r="D11" s="10" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>4:34/km</t>
         </is>
@@ -1070,7 +1111,8 @@
       </c>
       <c r="B12" s="12" t="inlineStr"/>
       <c r="C12" s="12" t="inlineStr"/>
-      <c r="D12" s="13" t="inlineStr"/>
+      <c r="D12" s="12" t="inlineStr"/>
+      <c r="E12" s="13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
@@ -1079,494 +1121,484 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
+        <is>
+          <t>Wings for Life World Run: Start 13:00 Uhr bei Schloss Schönbrunn; das Catcher Car startet 30 Minuten später mit 12,9 → 14,5 → 16,1 km/h. Bei 5:44/km liegt die Einholung rechnerisch bei rund 19,33 km.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Tests</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
-      <c r="J16" s="3" t="n"/>
-      <c r="K16" s="4" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+      <c r="G17" s="3" t="n"/>
+      <c r="H17" s="3" t="n"/>
+      <c r="I17" s="3" t="n"/>
+      <c r="J17" s="3" t="n"/>
+      <c r="K17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Merkmal</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>Test 1</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
         <is>
           <t>Test 2</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>Test 3</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>Test 4</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>Test 5</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
         <is>
           <t>Test 6</t>
         </is>
       </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>Test 7</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Test 8</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Test 9</t>
         </is>
       </c>
-      <c r="K17" s="7" t="inlineStr">
+      <c r="K18" s="7" t="inlineStr">
         <is>
           <t>Test 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="8" t="inlineStr">
-        <is>
-          <t>Woche</t>
-        </is>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 4</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 8</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 13</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 20</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 22</t>
-        </is>
-      </c>
-      <c r="G18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 29</t>
-        </is>
-      </c>
-      <c r="H18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 31</t>
-        </is>
-      </c>
-      <c r="I18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 39</t>
-        </is>
-      </c>
-      <c r="J18" s="9" t="inlineStr">
-        <is>
-          <t>Woche 44</t>
-        </is>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
-        <is>
-          <t>Woche 49</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Woche</t>
         </is>
       </c>
       <c r="B19" s="9" t="inlineStr">
         <is>
-          <t>18.10.2026</t>
+          <t>Woche 4</t>
         </is>
       </c>
       <c r="C19" s="9" t="inlineStr">
         <is>
-          <t>15.11.2026</t>
+          <t>Woche 8</t>
         </is>
       </c>
       <c r="D19" s="9" t="inlineStr">
         <is>
-          <t>20.12.2026</t>
+          <t>Woche 13</t>
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr">
         <is>
-          <t>07.02.2027</t>
+          <t>Woche 20</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
         <is>
-          <t>21.02.2027</t>
+          <t>Woche 22</t>
         </is>
       </c>
       <c r="G19" s="9" t="inlineStr">
         <is>
-          <t>11.04.2027</t>
+          <t>Woche 29</t>
         </is>
       </c>
       <c r="H19" s="9" t="inlineStr">
         <is>
-          <t>25.04.2027</t>
+          <t>Woche 31</t>
         </is>
       </c>
       <c r="I19" s="9" t="inlineStr">
         <is>
-          <t>20.06.2027</t>
+          <t>Woche 39</t>
         </is>
       </c>
       <c r="J19" s="9" t="inlineStr">
         <is>
-          <t>25.07.2027</t>
+          <t>Woche 44</t>
         </is>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>29.08.2027</t>
+          <t>Woche 49</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t>Teil 1</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>5 km locker @ 7:45</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>3 km zügig @ 5:35</t>
-        </is>
-      </c>
-      <c r="D20" s="15" t="inlineStr">
-        <is>
-          <t>5 km zügig @ 5:45</t>
-        </is>
-      </c>
-      <c r="E20" s="15" t="inlineStr">
-        <is>
-          <t>5,7 km Test @ 5:15</t>
-        </is>
-      </c>
-      <c r="F20" s="15" t="inlineStr">
-        <is>
-          <t>10 km locker @ 7:05</t>
-        </is>
-      </c>
-      <c r="G20" s="15" t="inlineStr">
-        <is>
-          <t>20 km locker @ 7:05</t>
-        </is>
-      </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>20 km locker @ 7:05</t>
-        </is>
-      </c>
-      <c r="I20" s="15" t="inlineStr">
-        <is>
-          <t>5,7 km Test @ 5:10</t>
-        </is>
-      </c>
-      <c r="J20" s="15" t="inlineStr">
-        <is>
-          <t>5,7 km Test @ 4:47</t>
-        </is>
-      </c>
-      <c r="K20" s="16" t="inlineStr">
-        <is>
-          <t>5,7 km Test @ 4:40</t>
+          <t>Datum</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="inlineStr">
+        <is>
+          <t>18.10.2026</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>15.11.2026</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>20.12.2026</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>07.02.2027</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>21.02.2027</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>11.04.2027</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>25.04.2027</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>20.06.2027</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>25.07.2027</t>
+        </is>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>29.08.2027</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
         <is>
-          <t>Teil 2</t>
+          <t>Teil 1</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5 km locker @ 7:45</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>3 km zügig @ 5:35</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5 km zügig @ 5:45</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5,7 km Test @ 5:15</t>
         </is>
       </c>
       <c r="F21" s="15" t="inlineStr">
         <is>
-          <t>10 km @ 5:41</t>
+          <t>10 km locker @ 7:05</t>
         </is>
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>8 km @ 6:24</t>
+          <t>20 km locker @ 7:05</t>
         </is>
       </c>
       <c r="H21" s="15" t="inlineStr">
         <is>
-          <t>10 km @ 6:24</t>
+          <t>20 km locker @ 7:05</t>
         </is>
       </c>
       <c r="I21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5,7 km Test @ 5:10</t>
         </is>
       </c>
       <c r="J21" s="15" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5,7 km Test @ 4:47</t>
         </is>
       </c>
       <c r="K21" s="16" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>5,7 km Test @ 4:40</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>Gesamt</t>
-        </is>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>5 km</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>3 km</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>5 km</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>5,7 km</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>20 km</t>
-        </is>
-      </c>
-      <c r="G22" s="9" t="inlineStr">
-        <is>
-          <t>28 km</t>
-        </is>
-      </c>
-      <c r="H22" s="9" t="inlineStr">
-        <is>
-          <t>30 km</t>
-        </is>
-      </c>
-      <c r="I22" s="9" t="inlineStr">
-        <is>
-          <t>5,7 km</t>
-        </is>
-      </c>
-      <c r="J22" s="9" t="inlineStr">
-        <is>
-          <t>5,7 km</t>
-        </is>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
-        <is>
-          <t>5,7 km</t>
+          <t>Teil 2</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F22" s="15" t="inlineStr">
+        <is>
+          <t>10 km @ 5:41</t>
+        </is>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>8 km @ 6:24</t>
+        </is>
+      </c>
+      <c r="H22" s="15" t="inlineStr">
+        <is>
+          <t>10 km @ 6:24</t>
+        </is>
+      </c>
+      <c r="I22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="15" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="16" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>Zielwert</t>
-        </is>
-      </c>
-      <c r="B23" s="15" t="inlineStr">
-        <is>
-          <t>38:45</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>16:45</t>
-        </is>
-      </c>
-      <c r="D23" s="15" t="inlineStr">
-        <is>
-          <t>28:45</t>
-        </is>
-      </c>
-      <c r="E23" s="15" t="inlineStr">
-        <is>
-          <t>29:56 (5:15/km)</t>
-        </is>
-      </c>
-      <c r="F23" s="15" t="inlineStr">
-        <is>
-          <t>10-km-Teil in 56:50</t>
-        </is>
-      </c>
-      <c r="G23" s="15" t="inlineStr">
-        <is>
-          <t>8-km-Teil in 51:12</t>
-        </is>
-      </c>
-      <c r="H23" s="15" t="inlineStr">
-        <is>
-          <t>10-km-Teil in 64:00</t>
-        </is>
-      </c>
-      <c r="I23" s="15" t="inlineStr">
-        <is>
-          <t>29:27</t>
-        </is>
-      </c>
-      <c r="J23" s="15" t="inlineStr">
-        <is>
-          <t>27:16 (4:47/km)</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
-        <is>
-          <t>26:38 (4:40/km)</t>
+          <t>Gesamt</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="inlineStr">
+        <is>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>3 km</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>5 km</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>5,7 km</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>20 km</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>28 km</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>30 km</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>5,7 km</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>5,7 km</t>
+        </is>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>5,7 km</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
+          <t>Zielwert</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>38:45</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
+          <t>28:45</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>29:56 (5:15/km)</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>10-km-Teil in 56:50</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>8-km-Teil in 51:12</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>10-km-Teil in 64:00</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>29:27</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>27:16 (4:47/km)</t>
+        </is>
+      </c>
+      <c r="K24" s="16" t="inlineStr">
+        <is>
+          <t>26:38 (4:40/km)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
           <t>Ist-Zeit</t>
         </is>
       </c>
-      <c r="B24" s="17" t="inlineStr"/>
-      <c r="C24" s="17" t="inlineStr"/>
-      <c r="D24" s="17" t="inlineStr"/>
-      <c r="E24" s="17" t="inlineStr"/>
-      <c r="F24" s="17" t="inlineStr"/>
-      <c r="G24" s="17" t="inlineStr"/>
-      <c r="H24" s="17" t="inlineStr"/>
-      <c r="I24" s="17" t="inlineStr"/>
-      <c r="J24" s="17" t="inlineStr"/>
-      <c r="K24" s="18" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="B25" s="17" t="inlineStr"/>
+      <c r="C25" s="17" t="inlineStr"/>
+      <c r="D25" s="17" t="inlineStr"/>
+      <c r="E25" s="17" t="inlineStr"/>
+      <c r="F25" s="17" t="inlineStr"/>
+      <c r="G25" s="17" t="inlineStr"/>
+      <c r="H25" s="17" t="inlineStr"/>
+      <c r="I25" s="17" t="inlineStr"/>
+      <c r="J25" s="17" t="inlineStr"/>
+      <c r="K25" s="18" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Gefühl</t>
         </is>
       </c>
-      <c r="B25" s="19" t="inlineStr"/>
-      <c r="C25" s="19" t="inlineStr"/>
-      <c r="D25" s="19" t="inlineStr"/>
-      <c r="E25" s="19" t="inlineStr"/>
-      <c r="F25" s="19" t="inlineStr"/>
-      <c r="G25" s="19" t="inlineStr"/>
-      <c r="H25" s="19" t="inlineStr"/>
-      <c r="I25" s="19" t="inlineStr"/>
-      <c r="J25" s="19" t="inlineStr"/>
-      <c r="K25" s="20" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr"/>
+      <c r="C26" s="19" t="inlineStr"/>
+      <c r="D26" s="19" t="inlineStr"/>
+      <c r="E26" s="19" t="inlineStr"/>
+      <c r="F26" s="19" t="inlineStr"/>
+      <c r="G26" s="19" t="inlineStr"/>
+      <c r="H26" s="19" t="inlineStr"/>
+      <c r="I26" s="19" t="inlineStr"/>
+      <c r="J26" s="19" t="inlineStr"/>
+      <c r="K26" s="20" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>Hinweise</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
-      <c r="J27" s="3" t="n"/>
-      <c r="K27" s="4" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>Lauftage: Montag kurz · Mittwoch kurz + Qualität · Freitag langer Lauf · Sa/So frei.</t>
-        </is>
-      </c>
-      <c r="B28" s="22" t="n"/>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
-      <c r="F28" s="22" t="n"/>
-      <c r="G28" s="22" t="n"/>
-      <c r="H28" s="22" t="n"/>
-      <c r="I28" s="22" t="n"/>
-      <c r="J28" s="22" t="n"/>
-      <c r="K28" s="23" t="n"/>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="4" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
-          <t>Wettkämpfe und Tests stehen an ihrem festen Datum in der Spalte Wettkampf/Test und ersetzen in dieser Woche den Freitagslauf.</t>
+          <t>Lauftage: Montag kurz · Mittwoch kurz + Qualität · Freitag langer Lauf · Sa/So frei.</t>
         </is>
       </c>
       <c r="B29" s="22" t="n"/>
@@ -1583,7 +1615,7 @@
     <row r="30">
       <c r="A30" s="21" t="inlineStr">
         <is>
-          <t>Blutwerte (Ferritin, B12, Vitamin D) vor Trainingsbeginn ärztlich checken lassen.</t>
+          <t>Wettkämpfe und Tests stehen an ihrem festen Datum in der Spalte Wettkampf/Test und ersetzen in dieser Woche den Freitagslauf.</t>
         </is>
       </c>
       <c r="B30" s="22" t="n"/>
@@ -1600,7 +1632,7 @@
     <row r="31">
       <c r="A31" s="21" t="inlineStr">
         <is>
-          <t>Dieser Plan ist kein Ersatz für ärztlichen Rat.</t>
+          <t>Blutwerte (Ferritin, B12, Vitamin D) vor Trainingsbeginn ärztlich checken lassen.</t>
         </is>
       </c>
       <c r="B31" s="22" t="n"/>
@@ -1617,7 +1649,7 @@
     <row r="32">
       <c r="A32" s="21" t="inlineStr">
         <is>
-          <t>Gelb hinterlegte Zellen sind zum Eintragen: Ist-Zeit und Gefühl.</t>
+          <t>Dieser Plan ist kein Ersatz für ärztlichen Rat.</t>
         </is>
       </c>
       <c r="B32" s="22" t="n"/>
@@ -1634,7 +1666,7 @@
     <row r="33">
       <c r="A33" s="21" t="inlineStr">
         <is>
-          <t>Beispiel Ist-Zeit: 28:32 · Beispiel Gefühl: locker, Beine ab km 8 schwer</t>
+          <t>Gelb hinterlegte Zellen sind zum Eintragen: Ist-Zeit und Gefühl.</t>
         </is>
       </c>
       <c r="B33" s="22" t="n"/>
@@ -1651,7 +1683,7 @@
     <row r="34">
       <c r="A34" s="21" t="inlineStr">
         <is>
-          <t>Traumziele bleiben als Anzeige stehen; das Training ist auf die Einschätzung kalibriert.</t>
+          <t>Beispiel Ist-Zeit: 28:32 · Beispiel Gefühl: locker, Beine ab km 8 schwer</t>
         </is>
       </c>
       <c r="B34" s="22" t="n"/>
@@ -1666,37 +1698,55 @@
       <c r="K34" s="23" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="24" t="inlineStr">
+      <c r="A35" s="21" t="inlineStr">
+        <is>
+          <t>Traumziele bleiben als Anzeige stehen; das Training ist auf die Einschätzung kalibriert.</t>
+        </is>
+      </c>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+      <c r="F35" s="22" t="n"/>
+      <c r="G35" s="22" t="n"/>
+      <c r="H35" s="22" t="n"/>
+      <c r="I35" s="22" t="n"/>
+      <c r="J35" s="22" t="n"/>
+      <c r="K35" s="23" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="24" t="inlineStr">
         <is>
           <t>Supplements stehen ausschließlich in der Zeile Supplements, nicht bei den Lebensmitteln.</t>
         </is>
       </c>
-      <c r="B35" s="25" t="n"/>
-      <c r="C35" s="25" t="n"/>
-      <c r="D35" s="25" t="n"/>
-      <c r="E35" s="25" t="n"/>
-      <c r="F35" s="25" t="n"/>
-      <c r="G35" s="25" t="n"/>
-      <c r="H35" s="25" t="n"/>
-      <c r="I35" s="25" t="n"/>
-      <c r="J35" s="25" t="n"/>
-      <c r="K35" s="26" t="n"/>
+      <c r="B36" s="25" t="n"/>
+      <c r="C36" s="25" t="n"/>
+      <c r="D36" s="25" t="n"/>
+      <c r="E36" s="25" t="n"/>
+      <c r="F36" s="25" t="n"/>
+      <c r="G36" s="25" t="n"/>
+      <c r="H36" s="25" t="n"/>
+      <c r="I36" s="25" t="n"/>
+      <c r="J36" s="25" t="n"/>
+      <c r="K36" s="26" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A34:K34"/>
     <mergeCell ref="A35:K35"/>
     <mergeCell ref="A30:K30"/>
+    <mergeCell ref="A15:K15"/>
     <mergeCell ref="A29:K29"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A16:K16"/>
     <mergeCell ref="A33:K33"/>
     <mergeCell ref="A28:K28"/>
     <mergeCell ref="A32:K32"/>
+    <mergeCell ref="A36:K36"/>
     <mergeCell ref="A14:K14"/>
+    <mergeCell ref="A31:K31"/>
     <mergeCell ref="A1:K1"/>
-    <mergeCell ref="A27:K27"/>
-    <mergeCell ref="A31:K31"/>
+    <mergeCell ref="A17:K17"/>
+    <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>